<commit_message>
Add resource calculator Excel and analysis plan
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/resource-calculator-platform-release-1.3.0.xlsx
+++ b/resource-calculator-platform-release-1.3.0.xlsx
@@ -549,7 +549,7 @@
     <numFmt numFmtId="180" formatCode="0.0"/>
     <numFmt numFmtId="181" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="48">
+  <fonts count="47">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -566,13 +566,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <i/>
       <sz val="10"/>
       <color theme="1"/>
@@ -855,8 +848,7 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
-      <charset val="1"/>
-      <scheme val="minor"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="9"/>
@@ -865,27 +857,28 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="9"/>
+      <name val="Tahoma"/>
+      <charset val="134"/>
+    </font>
+    <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <name val="Tahoma"/>
-      <charset val="134"/>
+      <charset val="1"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+      <scheme val="major"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <charset val="1"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <charset val="1"/>
-      <scheme val="major"/>
     </font>
     <font>
       <sz val="10"/>
@@ -895,7 +888,7 @@
       <scheme val="major"/>
     </font>
   </fonts>
-  <fills count="46">
+  <fills count="44">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1030,12 +1023,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="4" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -1079,12 +1066,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1747,109 +1728,115 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="21" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="21" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="21" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="21" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="21" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="20" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="20" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="20" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="20" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="20" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="40" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="40" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="41" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="41" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="41" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="42" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="16" borderId="43" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="17" borderId="44" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="17" borderId="43" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="18" borderId="45" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="46" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="47" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="42" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="16" borderId="43" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="17" borderId="44" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="17" borderId="43" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="18" borderId="45" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="46" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="47" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="39" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="39" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="39" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="39" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="39" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1858,10 +1845,10 @@
     <xf numFmtId="0" fontId="39" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="38" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="39" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1870,10 +1857,10 @@
     <xf numFmtId="0" fontId="39" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="38" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="39" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1882,13 +1869,7 @@
     <xf numFmtId="0" fontId="39" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="43" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="45" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="38" fillId="43" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1897,51 +1878,51 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="6" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="5" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="6" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="5" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1950,95 +1931,95 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="6" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="9" fontId="5" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="6" fillId="5" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="5" fillId="5" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="9" fillId="8" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="9" fillId="8" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="8" fillId="8" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="8" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
@@ -2047,370 +2028,370 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="9" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="9" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="180" fontId="6" fillId="6" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="6" fillId="6" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="6" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="180" fontId="5" fillId="6" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="5" fillId="6" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="5" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="180" fontId="6" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="6" fillId="6" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="180" fontId="5" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="5" fillId="6" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="180" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="6" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="12" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="180" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="5" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="12" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="10" fillId="12" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="10" fillId="12" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="10" fillId="12" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="9" fillId="12" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="12" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="12" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="6" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="5" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="6" fillId="3" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="5" fillId="3" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="6" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="180" fontId="6" fillId="4" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="3" fontId="5" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="180" fontId="5" fillId="4" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="181" fontId="6" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="181" fontId="5" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="6" fillId="5" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="6" fillId="5" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="5" fillId="5" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="5" fillId="5" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="9" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="9" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="15" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="180" fontId="15" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="180" fontId="14" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="180" fontId="15" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="180" fontId="14" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="15" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="14" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="180" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="180" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="4" fillId="12" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="3" fillId="12" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="4" fillId="12" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="3" fillId="12" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="6" fillId="13" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="3" fontId="5" fillId="13" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="6" fillId="13" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="5" fillId="13" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="6" fillId="13" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="5" fillId="13" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="14" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="14" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="1" fillId="14" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2419,22 +2400,22 @@
     <xf numFmtId="3" fontId="1" fillId="14" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2800,7 +2781,7 @@
       <c r="A12" s="185"/>
       <c r="B12" s="119"/>
     </row>
-    <row r="13" customFormat="1" ht="13.95"/>
+    <row r="13" ht="13.95"/>
     <row r="14" ht="13.5" customHeight="1" spans="1:13">
       <c r="A14" s="186" t="s">
         <v>10</v>
@@ -2836,23 +2817,23 @@
       </c>
       <c r="B15" s="119">
         <f>'Registrations Upload &amp; SyncData'!B17</f>
-        <v>25000000</v>
+        <v>250000</v>
       </c>
       <c r="C15" s="133">
         <f>'Registrations Upload &amp; SyncData'!B19</f>
-        <v>8334</v>
+        <v>84</v>
       </c>
       <c r="D15" s="133">
         <f>'Registrations Upload &amp; SyncData'!E29</f>
-        <v>23145</v>
+        <v>250</v>
       </c>
       <c r="E15" s="133">
         <f>'Registrations Upload &amp; SyncData'!F29</f>
-        <v>62502</v>
+        <v>674</v>
       </c>
       <c r="F15" s="133">
         <f>'Registrations Upload &amp; SyncData'!G29</f>
-        <v>9277</v>
+        <v>102</v>
       </c>
       <c r="G15" s="192"/>
       <c r="H15" s="192"/>
@@ -2902,15 +2883,15 @@
       <c r="C17" s="194"/>
       <c r="D17" s="195">
         <f>SUM(D15:D16)</f>
-        <v>23362</v>
+        <v>467</v>
       </c>
       <c r="E17" s="195">
         <f>SUM(E15:E16)</f>
-        <v>63199</v>
+        <v>1371</v>
       </c>
       <c r="F17" s="196">
         <f>SUM(F15:F16)</f>
-        <v>9364</v>
+        <v>189</v>
       </c>
       <c r="G17" s="192"/>
       <c r="H17" s="192"/>
@@ -2939,7 +2920,7 @@
       </c>
       <c r="B19" s="199">
         <f>'Registrations Upload &amp; SyncData'!B27</f>
-        <v>1</v>
+        <v>400</v>
       </c>
       <c r="C19" s="20"/>
       <c r="D19" s="20"/>
@@ -3025,7 +3006,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="111">
-        <v>1000000</v>
+        <v>100000000</v>
       </c>
       <c r="C7" s="12" t="s">
         <v>24</v>
@@ -3038,7 +3019,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="115">
-        <v>50000</v>
+        <v>5000</v>
       </c>
       <c r="C8" s="116"/>
       <c r="D8" s="112"/>
@@ -3049,7 +3030,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="118">
-        <v>500</v>
+        <v>50</v>
       </c>
       <c r="C9" s="116"/>
       <c r="D9" s="112"/>
@@ -3104,7 +3085,7 @@
       <c r="G14" s="123"/>
     </row>
     <row r="15" ht="13.95"/>
-    <row r="16" spans="1:2">
+    <row r="16" ht="13.95" spans="1:2">
       <c r="A16" s="36" t="s">
         <v>30</v>
       </c>
@@ -3118,7 +3099,7 @@
       </c>
       <c r="B17" s="126">
         <f>B8*B9</f>
-        <v>25000000</v>
+        <v>250000</v>
       </c>
     </row>
     <row r="18" customFormat="1" spans="1:2">
@@ -3127,7 +3108,7 @@
       </c>
       <c r="B18" s="126">
         <f>B17*B14</f>
-        <v>30000000</v>
+        <v>300000</v>
       </c>
     </row>
     <row r="19" ht="13.95" spans="1:2">
@@ -3136,13 +3117,13 @@
       </c>
       <c r="B19" s="128">
         <f>CEILING(B18/B13/3600,1)</f>
-        <v>8334</v>
+        <v>84</v>
       </c>
     </row>
     <row r="20" ht="13.95" spans="10:10">
       <c r="J20" s="9"/>
     </row>
-    <row r="21" spans="1:2">
+    <row r="21" ht="13.95" spans="1:2">
       <c r="A21" s="36" t="s">
         <v>34</v>
       </c>
@@ -3168,17 +3149,17 @@
       </c>
       <c r="B24" s="135">
         <f>CEILING(B19/B22,1)</f>
-        <v>371</v>
-      </c>
-    </row>
-    <row r="26" customFormat="1" ht="13.95"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26" ht="13.95"/>
     <row r="27" customFormat="1" ht="21.15" spans="1:2">
       <c r="A27" s="47" t="s">
         <v>20</v>
       </c>
       <c r="B27" s="136">
         <f>CEILING(B7/B17,1)</f>
-        <v>1</v>
+        <v>400</v>
       </c>
     </row>
     <row r="28" customFormat="1" ht="13.95" spans="1:7">
@@ -3205,15 +3186,15 @@
       <c r="D29" s="48"/>
       <c r="E29" s="49">
         <f>E53</f>
-        <v>23145</v>
+        <v>250</v>
       </c>
       <c r="F29" s="49">
         <f>F53</f>
-        <v>62502</v>
+        <v>674</v>
       </c>
       <c r="G29" s="50">
         <f>G53</f>
-        <v>9277</v>
+        <v>102</v>
       </c>
     </row>
     <row r="30" customFormat="1" ht="20.4" spans="1:7">
@@ -3316,15 +3297,15 @@
       </c>
       <c r="E37" s="146">
         <f>$G37*B37</f>
-        <v>742</v>
+        <v>8</v>
       </c>
       <c r="F37" s="147">
         <f>$G37*C37</f>
-        <v>742</v>
+        <v>8</v>
       </c>
       <c r="G37" s="148">
         <f t="shared" ref="G37:G45" si="0">$B$24*D37</f>
-        <v>742</v>
+        <v>8</v>
       </c>
     </row>
     <row r="38" spans="1:7">
@@ -3342,15 +3323,15 @@
       </c>
       <c r="E38" s="149">
         <f t="shared" ref="E38:E46" si="1">$G38*B38</f>
-        <v>519.4</v>
+        <v>5.6</v>
       </c>
       <c r="F38" s="150">
         <f t="shared" ref="F38:F47" si="2">$G38*C38</f>
-        <v>1113</v>
+        <v>12</v>
       </c>
       <c r="G38" s="151">
         <f t="shared" si="0"/>
-        <v>742</v>
+        <v>8</v>
       </c>
     </row>
     <row r="39" spans="1:7">
@@ -3368,15 +3349,15 @@
       </c>
       <c r="E39" s="149">
         <f t="shared" si="1"/>
-        <v>742</v>
+        <v>8</v>
       </c>
       <c r="F39" s="150">
         <f t="shared" si="2"/>
-        <v>3710</v>
+        <v>40</v>
       </c>
       <c r="G39" s="151">
         <f t="shared" si="0"/>
-        <v>742</v>
+        <v>8</v>
       </c>
     </row>
     <row r="40" spans="1:7">
@@ -3394,15 +3375,15 @@
       </c>
       <c r="E40" s="149">
         <f t="shared" si="1"/>
-        <v>2226</v>
+        <v>24</v>
       </c>
       <c r="F40" s="150">
         <f t="shared" si="2"/>
-        <v>2782.5</v>
+        <v>30</v>
       </c>
       <c r="G40" s="151">
         <f t="shared" si="0"/>
-        <v>1113</v>
+        <v>12</v>
       </c>
     </row>
     <row r="41" customFormat="1" spans="1:7">
@@ -3420,15 +3401,15 @@
       </c>
       <c r="E41" s="149">
         <f t="shared" si="1"/>
-        <v>2968</v>
+        <v>32</v>
       </c>
       <c r="F41" s="150">
         <f t="shared" si="2"/>
-        <v>8904</v>
+        <v>96</v>
       </c>
       <c r="G41" s="151">
         <f t="shared" si="0"/>
-        <v>1484</v>
+        <v>16</v>
       </c>
     </row>
     <row r="42" customFormat="1" spans="1:7">
@@ -3446,15 +3427,15 @@
       </c>
       <c r="E42" s="149">
         <f t="shared" si="1"/>
-        <v>371</v>
+        <v>4</v>
       </c>
       <c r="F42" s="150">
         <f t="shared" si="2"/>
-        <v>1669.5</v>
+        <v>18</v>
       </c>
       <c r="G42" s="151">
         <f t="shared" si="0"/>
-        <v>742</v>
+        <v>8</v>
       </c>
     </row>
     <row r="43" customFormat="1" spans="1:7">
@@ -3472,15 +3453,15 @@
       </c>
       <c r="E43" s="149">
         <f t="shared" si="1"/>
-        <v>1484</v>
+        <v>16</v>
       </c>
       <c r="F43" s="150">
         <f t="shared" si="2"/>
-        <v>3710</v>
+        <v>40</v>
       </c>
       <c r="G43" s="151">
         <f t="shared" si="0"/>
-        <v>742</v>
+        <v>8</v>
       </c>
     </row>
     <row r="44" customFormat="1" spans="1:7">
@@ -3498,15 +3479,15 @@
       </c>
       <c r="E44" s="149">
         <f t="shared" si="1"/>
-        <v>1113</v>
+        <v>12</v>
       </c>
       <c r="F44" s="150">
         <f t="shared" si="2"/>
-        <v>5565</v>
+        <v>60</v>
       </c>
       <c r="G44" s="151">
         <f t="shared" si="0"/>
-        <v>1113</v>
+        <v>12</v>
       </c>
     </row>
     <row r="45" spans="1:7">
@@ -3524,15 +3505,15 @@
       </c>
       <c r="E45" s="149">
         <f t="shared" si="1"/>
-        <v>3710</v>
+        <v>40</v>
       </c>
       <c r="F45" s="150">
         <f t="shared" si="2"/>
-        <v>9275</v>
+        <v>100</v>
       </c>
       <c r="G45" s="151">
         <f t="shared" si="0"/>
-        <v>1855</v>
+        <v>20</v>
       </c>
     </row>
     <row r="46" spans="1:8">
@@ -3581,15 +3562,15 @@
       <c r="D48" s="158"/>
       <c r="E48" s="159">
         <f>SUM(E37:E47)</f>
-        <v>13875.4</v>
+        <v>149.6</v>
       </c>
       <c r="F48" s="158">
         <f>SUM(F37:F47)</f>
-        <v>37471</v>
+        <v>404</v>
       </c>
       <c r="G48" s="160">
         <f>SUM(G37:G47)</f>
-        <v>9277</v>
+        <v>102</v>
       </c>
     </row>
     <row r="49" ht="13.95" spans="1:7">
@@ -3612,11 +3593,11 @@
       <c r="D50" s="165"/>
       <c r="E50" s="166">
         <f t="shared" ref="E50:F50" si="4">E48*0.2</f>
-        <v>2775.08</v>
+        <v>29.92</v>
       </c>
       <c r="F50" s="166">
         <f t="shared" si="4"/>
-        <v>7494.2</v>
+        <v>80.8</v>
       </c>
       <c r="G50" s="167"/>
     </row>
@@ -3629,11 +3610,11 @@
       <c r="D51" s="165"/>
       <c r="E51" s="166">
         <f>ROUND((E48+E50)*0.3,2)</f>
-        <v>4995.14</v>
+        <v>53.86</v>
       </c>
       <c r="F51" s="166">
         <f>(F48+F50)*0.3</f>
-        <v>13489.56</v>
+        <v>145.44</v>
       </c>
       <c r="G51" s="167"/>
     </row>
@@ -3646,11 +3627,11 @@
       <c r="D52" s="165"/>
       <c r="E52" s="166">
         <f t="shared" ref="E52:F52" si="5">ROUND((E51*0.3),2)</f>
-        <v>1498.54</v>
+        <v>16.16</v>
       </c>
       <c r="F52" s="166">
         <f t="shared" si="5"/>
-        <v>4046.87</v>
+        <v>43.63</v>
       </c>
       <c r="G52" s="167"/>
     </row>
@@ -3663,15 +3644,15 @@
       <c r="D53" s="169"/>
       <c r="E53" s="170">
         <f>CEILING((SUM(E48:E52)),1)</f>
-        <v>23145</v>
+        <v>250</v>
       </c>
       <c r="F53" s="170">
         <f>CEILING(SUM(F48:F52),1)</f>
-        <v>62502</v>
+        <v>674</v>
       </c>
       <c r="G53" s="171">
         <f>SUM(G37:G47)</f>
-        <v>9277</v>
+        <v>102</v>
       </c>
     </row>
     <row r="54" spans="1:8">

</xml_diff>